<commit_message>
Add real drywall/ceiling repair purchase data to Budget Tracker
Logs the actual receipt (PO confirmed for 1464 Sunrise Pkwy, paid via the
zero-balance Home Depot card per Juan's instruction): joint compound,
drywall tape, corner tape, and grout compound. Grand Total formula
updated to include the new rows.
</commit_message>
<xml_diff>
--- a/projects/1464-sunrise-pkwy-tracker.xlsx
+++ b/projects/1464-sunrise-pkwy-tracker.xlsx
@@ -3042,7 +3042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3226,29 +3226,177 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Living Room/Ceiling</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Joint compound, 18 lb Fast Set (Custom Building Products)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Building supply (San Rafael, CA) - HD card</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>17.48</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" s="6">
+        <f>D7*E7</f>
+        <v/>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Ceiling/drywall repair</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Living Room/Ceiling</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Vinyl drywall tape (Dryvit)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Building supply (San Rafael, CA) - HD card</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>9.93</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="6">
+        <f>D8*E8</f>
+        <v/>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Living Room/Ceiling</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>FibaTape self-adhesive mesh drywall joint tape (Cofair ADFORS)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Building supply (San Rafael, CA) - HD card</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>15.98</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" s="6">
+        <f>D9*E9</f>
+        <v/>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Living Room/Ceiling</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Flexible paper corner tape, 100 ft (OX)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Building supply (San Rafael, CA) - HD card</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>21.26</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="6">
+        <f>D10*E10</f>
+        <v/>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Living Room/Ceiling</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Grout Boost compound (Custom Building Products)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Building supply (San Rafael, CA) - HD card</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>15.11</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="F11" s="6">
+        <f>D11*E11</f>
+        <v/>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>$2.32 discount applied on receipt</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="F8" s="6">
-        <f>SUM(F2:F6)</f>
+      <c r="F13" s="6">
+        <f>SUM(F2:F11)</f>
         <v/>
       </c>
-      <c r="G8" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mark garage door as approved
</commit_message>
<xml_diff>
--- a/projects/1464-sunrise-pkwy-tracker.xlsx
+++ b/projects/1464-sunrise-pkwy-tracker.xlsx
@@ -2123,17 +2123,17 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Garage door (exterior) needs replacement; kitchen-&gt;garage door wood, dirty, needs repaint</t>
+          <t>Garage door (exterior) APPROVED - Precision, Lincoln 3138, white flush-panel, $2,273.75; kitchen-&gt;garage door wood, dirty, needs repaint</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>Replace</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Is garage door replacement authorized under the permit ('repairing siding' only)?</t>
+          <t>Color conflicts with dark-exterior direction - reconcile at Monday's meeting</t>
         </is>
       </c>
     </row>
@@ -3021,7 +3021,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Answered</t>
         </is>
       </c>
     </row>

</xml_diff>